<commit_message>
Update code and slides
</commit_message>
<xml_diff>
--- a/data/schedule/schedule.xlsx
+++ b/data/schedule/schedule.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="33">
   <si>
     <t>Date</t>
   </si>
@@ -68,6 +68,15 @@
   </si>
   <si>
     <t>Effects of Monetary Policy · Geometries</t>
+  </si>
+  <si>
+    <t>03_effects</t>
+  </si>
+  <si>
+    <t>03_geometries.R</t>
+  </si>
+  <si>
+    <t>03_geometries.RData</t>
   </si>
   <si>
     <t>Quantitative Easing · Scales</t>
@@ -1343,9 +1352,15 @@
       <c r="D4" t="s" s="2">
         <v>18</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+      <c r="E4" t="s" s="2">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s" s="2">
+        <v>21</v>
+      </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
     </row>
@@ -1360,7 +1375,7 @@
         <v>10</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
@@ -1379,7 +1394,7 @@
         <v>10</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
@@ -1388,7 +1403,7 @@
         <v>2</v>
       </c>
       <c r="I6" t="s" s="2">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" ht="15.35" customHeight="1">
@@ -1402,7 +1417,7 @@
         <v>10</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
@@ -1421,7 +1436,7 @@
         <v>10</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
@@ -1430,7 +1445,7 @@
         <v>3</v>
       </c>
       <c r="I8" t="s" s="2">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" ht="15.35" customHeight="1">
@@ -1444,7 +1459,7 @@
         <v>10</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
@@ -1460,10 +1475,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
@@ -1472,7 +1487,7 @@
         <v>4</v>
       </c>
       <c r="I10" t="s" s="2">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" ht="15.35" customHeight="1">
@@ -1486,7 +1501,7 @@
         <v>10</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
@@ -1505,7 +1520,7 @@
         <v>10</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
@@ -1524,7 +1539,7 @@
         <v>10</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>

</xml_diff>

<commit_message>
Update slides for session 3
</commit_message>
<xml_diff>
--- a/data/schedule/schedule.xlsx
+++ b/data/schedule/schedule.xlsx
@@ -52,7 +52,7 @@
     <t>01_introduction</t>
   </si>
   <si>
-    <t>Monetary Regimes · Data handling</t>
+    <t>Money · Data handling</t>
   </si>
   <si>
     <t>02_money</t>
@@ -67,10 +67,10 @@
     <t>rstudio</t>
   </si>
   <si>
-    <t>Effects of Monetary Policy · Geometries</t>
-  </si>
-  <si>
-    <t>03_effects</t>
+    <t>Monetary Regimes · Geometries</t>
+  </si>
+  <si>
+    <t>03_regimes</t>
   </si>
   <si>
     <t>03_geometries.R</t>
@@ -82,13 +82,13 @@
     <t>Quantitative Easing · Scales</t>
   </si>
   <si>
-    <t>Financialization and Debt · Colors</t>
+    <t>Effects of Monetary Policy · Colors</t>
   </si>
   <si>
     <t>lines</t>
   </si>
   <si>
-    <t>tba · Labels</t>
+    <t>Financialization and Debt · Labels</t>
   </si>
   <si>
     <t>Introduction into data by OeNB</t>

</xml_diff>